<commit_message>
Course update: evidence pyramid, glossary, grading benchmarks, legal basics and Toolkit refreshed
Module folders 00 to 04 stay at their last published version until their rebuilt parts are approved.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XeVTcY3N2EX3kZsVA3PUfV
</commit_message>
<xml_diff>
--- a/resources/Co-Founder_Matchmaking_Assessment.xlsx
+++ b/resources/Co-Founder_Matchmaking_Assessment.xlsx
@@ -12,159 +12,159 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
-  <si>
-    <t>TUM VL – Co-Founder Assessment</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="77">
+  <si>
+    <t xml:space="preserve">Ambitious Entrepreneurship – Co-Founder Assessment</t>
   </si>
   <si>
     <t>Instructions</t>
   </si>
   <si>
-    <t>1. Copy this document -&gt; "File" -&gt; "Create Copy"</t>
-  </si>
-  <si>
-    <t>2. Take some time to fill out the fields as honestly as possible</t>
-  </si>
-  <si>
-    <t>3. Compare the answers with your potential co-founders</t>
-  </si>
-  <si>
-    <t>4. Discuss all the answers. Understand the why of yourself and your potential co-founder behind any match and any disagreement</t>
+    <t xml:space="preserve">1. Save your own copy of this file.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Answer every question alone and honestly, before you see anyone else's answers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Put your answers next to your potential co-founders' answers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Talk through every match and every gap, and ask why, for them and for yourself. Write what you agree into the Team sheet of your Student Toolkit.</t>
   </si>
   <si>
     <t>Operations</t>
   </si>
   <si>
-    <t>How many hours/week are you willing to work in general? For how long? What sounds good? What sounds like hell? Do you have different expectations for different phases of the company’s lifespan? (i.e. willing to work harder in the beginning)</t>
-  </si>
-  <si>
-    <t>Describe your personal working style. What tools and techniques do you use to keep yourself organised. How and how often do you like to take your breaks. How do you distribute off time over the week and over the year?</t>
-  </si>
-  <si>
-    <t>Describe what you consider good communication between peers. How do you give praise, what do you need to get to feel valued? What is bad communication, how does it affect your mood, and how can you get out of this state again?</t>
-  </si>
-  <si>
-    <t>How do you derive at your decisions? How long did it take you in the past? How did you handle differing oppinions with other people?</t>
-  </si>
-  <si>
-    <t>How do you prioritiese your work, your family, your health and other parts of your life? What unhealthy habits did you fall into in the past and what do you do to avoid it?</t>
-  </si>
-  <si>
-    <t>Reflect on a very stressful time in your life. What caused the stress? How did you handle it? How does it affect different parts of your life? How did you get out of it again?</t>
+    <t xml:space="preserve">How many hours a week do you want to work, and for how long can you keep that up? Which pace sounds great to you, and which sounds unbearable? Would you work harder in the first year than later?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How do you organise your work? Which tools and habits keep you on track, when do you take breaks, and how do you spread time off across a week and a year?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What does good communication between co-founders look like to you? How do you like to be recognised? What kind of communication drags you down, and how do you recover from it?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How do you make decisions, and how long do they usually take you? Think of a time you disagreed with someone close. What did you do?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How do you balance work, family, health and the rest of your life? Which unhealthy habits have you slipped into before, and what keeps you out of them now?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Think of the most stressful period you have lived through. What caused it, how did it show in your life, and what got you out of it?</t>
   </si>
   <si>
     <t>Hard factors</t>
   </si>
   <si>
-    <t>Is there anything I should know that may affect your time or legal status as a founder? (e.g. visa, green card, criminal record)</t>
-  </si>
-  <si>
-    <t>Will this company be your primary activity? Do you have any other time commitments?</t>
-  </si>
-  <si>
-    <t>What is your expected time commitment right now? How do you see that changing in the next 6 months? 2 years?</t>
-  </si>
-  <si>
-    <t>What is your life's plan. Are you planning on a family, getting back to school, doing something else eventually?</t>
+    <t xml:space="preserve">Is there anything that could limit your time or your legal ability to found a company, such as a visa, an employment contract or a non-compete?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Will this company be your main job? What else needs your time?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How many hours can you give right now, and how will that change in six months and in two years?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What are your plans for the next years outside the company, such as a family, more study or another career?</t>
   </si>
   <si>
     <t>Ambition</t>
   </si>
   <si>
-    <t>What are your plans for your next company? Do you want to bootstrap it, do you want to build a venture case. How much money do you think you'll need? How many people should be involved?</t>
-  </si>
-  <si>
-    <t>What does an ideal company exit look like to you? (i.e. “work on company for 1-2 years and sell for 7 figures” to “work for 10 + years, reach 9 figures in revenue, and IPO”)</t>
-  </si>
-  <si>
-    <t>How do you think about the timeframe and pace of success? Are you willing to take the longer path? How long is too long?</t>
-  </si>
-  <si>
-    <t>What does it take for you to feel free? What does it take for you to feel safe? Think of money, social status, control, opportunities, health and more.</t>
-  </si>
-  <si>
-    <t>Why do you want to start a company — in general, and in particular right now?</t>
-  </si>
-  <si>
-    <t>What number would you sell at? How would that change if you got extra liquidity from your existing positions?</t>
+    <t xml:space="preserve">Do you want to build a profitable business funded by its customers, or a venture-funded startup? How much money and how many people do you think it will take?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What would a great ending look like for you? Selling within a few years, or building for a decade or more and going public?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How long are you willing to wait for success? At what point would the road feel too long?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What do you need to feel free, and what do you need to feel safe? Think of money, status, control, options and health.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Why do you want to start a company at all, and why now?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At what price would you sell the company? Would that change if you already had money in the bank?</t>
   </si>
   <si>
     <t>Roles</t>
   </si>
   <si>
-    <t>What do we do if we find product/market fit, yet none of the founders are excited about that product?</t>
-  </si>
-  <si>
-    <t>What is the biggest project you are proud of to date? Why did you start it? What makes you proud? How did it end?</t>
-  </si>
-  <si>
-    <t>Is control or success more important? (i.e. Are you willing to step aside if the company is more likely to have a financially successful outcome or is it important for the founders to stay in control of the company’s destiny?)</t>
-  </si>
-  <si>
-    <t>Communication</t>
-  </si>
-  <si>
-    <t>How should founder equity be set? What’s your philosophy on an employee equity pool?</t>
-  </si>
-  <si>
-    <t>Under which circumstances can you be fired as a co-founder? Under which circumstances can you fire your co-founder?</t>
-  </si>
-  <si>
-    <t>What are your personal savings? How long can these support you? Would you invest your own money (ideally retaining higher equity in return)?</t>
-  </si>
-  <si>
-    <t>What is the minimum monthly salary you need to survive? To be comfortable? To feel like you've “made it?”</t>
-  </si>
-  <si>
-    <t>In case this becomes part of our partnership’s evolution, how would you go about handling a startup divorce? Who would leave and who would stay with the company?</t>
-  </si>
-  <si>
-    <t>What happens in the scenario where we aren’t growing? How would we diagnose the problem? How have each of our capabilities and approach contributed to growth failures in our pasts?</t>
-  </si>
-  <si>
-    <t>In every partnership, there are times when a partner might breed resentment if certain dissatisfactions don’t change over time. How would you deal with a situation like this?</t>
-  </si>
-  <si>
-    <t>How would you think about bringing on another cofounder in the future development of your company?</t>
+    <t xml:space="preserve">Suppose customers love what we build, but none of us is excited about it. What do we do?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which project are you proudest of so far? Why did you start it, what makes you proud, and how did it end?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which matters more to you, control or success? Would you step aside if someone else gave the company a better chance?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Money and exit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How should we split the founders' equity, and how much should we set aside for future employees?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When could a co-founder be asked to leave, you included? When would you ask a co-founder to leave?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How much savings do you have, and how many months will they last? Would you put your own money into the company, and should that earn you more equity?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What is the least you can live on per month? What would feel comfortable, and what would feel like success?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If we ever split up, how should that work? Who leaves, who stays, and what happens to the shares?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What do we do if the company stops growing? How do we find out why? What did each of us contribute when growth stalled in the past?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small frustrations can grow into resentment between partners. How would you raise one before it gets there?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Would you add another co-founder later? Under which conditions?</t>
   </si>
   <si>
     <t>Culture</t>
   </si>
   <si>
-    <t>What are the personal values that you would like to bring to a company? Describe them and what you would do to implement them.</t>
-  </si>
-  <si>
-    <t>What processes or techniques would you use to get the most out of your team? For example, how would you help them become better managers or achieve their goals?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How much of your time do you hope to spend either working or socializing with coworkers? How close or distant would you keep the relationship (i.e. Purely professional? We should all be best friends?) </t>
-  </si>
-  <si>
-    <t>How important is diversity &amp; inclusion? Concretely, how would you put that into action?</t>
+    <t xml:space="preserve">Which personal values do you want this company to live by, and how would you put each one into practice?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How would you help the people on your team grow, as managers or in reaching their own goals?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How much time do you want to spend with your colleagues, at work and outside it? Strictly professional, or close friends?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How much does a diverse and inclusive team matter to you, and what would you do about it in practice?</t>
   </si>
   <si>
     <t>Motivation</t>
   </si>
   <si>
-    <t>What interests you about ideas that you love? What makes you work long hours and put all your heart into it.</t>
-  </si>
-  <si>
-    <t>What markets do you like most and why? (B2B, B2C, Construction, Enterprise, ...)</t>
-  </si>
-  <si>
-    <t>Why are you a good addition to a founding team?</t>
-  </si>
-  <si>
-    <t>Who would you need as a mentor and why?</t>
-  </si>
-  <si>
-    <t>Source: Inspired from First Round and the Adoptions by Antler</t>
+    <t xml:space="preserve">What draws you to the ideas you love? What makes you work long hours on something with your whole heart?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which markets excite you most, and why? For example B2B, B2C, construction or enterprise software.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What do you bring to a founding team that others do not?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which mentor would you need, and why?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambitious Entrepreneurship · Dr. Bastian Burger</t>
   </si>
   <si>
     <t>Link to First Round Article</t>
   </si>
   <si>
-    <t>TUM VL – Founder Assessment – Roles</t>
+    <t xml:space="preserve">Ambitious Entrepreneurship – Co-Founder Assessment – Roles</t>
   </si>
   <si>
     <t>YOU</t>
@@ -182,34 +182,34 @@
     <t>Level of agreement</t>
   </si>
   <si>
-    <t>Roles &amp; responsibilites</t>
-  </si>
-  <si>
-    <t>How do you see your role changing as the company starts to scale? (Read the Review article on giving away your Legos.)</t>
-  </si>
-  <si>
-    <t>Who would be the CEO? Could this change over time?</t>
-  </si>
-  <si>
-    <t>Who would be in the press limelight? Always the entire team? One person in particular?</t>
-  </si>
-  <si>
-    <t>If your role becomes unavailable entirely (e.g. the board hires a professional CEO or an experienced executive), what would you want your new role to be?</t>
+    <t xml:space="preserve">Roles and responsibilities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How do you expect your role to change as the company grows? Which tasks would you hand over first?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Who should be CEO? Could that change over time?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Who should speak for the company in public? All of us, or one person?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If your role disappears, for example because the board hires an experienced CEO or executive, which role would you want instead?</t>
   </si>
   <si>
     <t>Who's in the lead?</t>
   </si>
   <si>
-    <t>Functional areas of expertise and responsibility - excercise</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Areas of Responsibility Exercise. Rank yourself in the following areas on a scale of 1=low 10=high. Then rate your passion in each of the above areas on a scale of none to high. (e.g. “I’m an 8 in sales, but hate it so none”). Note: Key is to decide this early-on for key functions for the business you are building. Less crucial functions can be decided or even shifted later. </t>
+    <t xml:space="preserve">Areas of expertise and responsibility, exercise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rate yourself from 1 (low) to 10 (high) in each area below, then rate how much you enjoy it, from none to high. For example, “I'm an 8 in sales, but I hate it, so none.” Settle early who owns the areas your business cannot run without. Others can wait or move later.</t>
   </si>
   <si>
     <t>Engineering</t>
   </si>
   <si>
-    <t>[Eg. Founder 1]</t>
+    <t xml:space="preserve">[e.g. Founder 1]</t>
   </si>
   <si>
     <t>Product</t>
@@ -236,7 +236,13 @@
     <t>Company Building</t>
   </si>
   <si>
-    <t>Domain knowledge (e.g. specific know-how)</t>
+    <t xml:space="preserve">Domain knowledge (specific know-how)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How you work</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tell us about a project that failed. What was your part in it, and what did you do differently afterwards?</t>
   </si>
 </sst>
 </file>
@@ -876,7 +882,7 @@
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="10" t="s">
-        <v>6</v>
+        <v>75</v>
       </c>
       <c r="C10" s="11"/>
       <c r="D10" s="12"/>
@@ -1152,7 +1158,7 @@
         <v>19</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>27</v>
+        <v>76</v>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="5"/>
@@ -1434,9 +1440,7 @@
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="1"/>
-      <c r="B62" s="23" t="s">
-        <v>49</v>
-      </c>
+      <c r="B62" s="23"/>
       <c r="C62" s="3"/>
       <c r="D62" s="4"/>
       <c r="E62" s="5"/>
@@ -1452,9 +1456,6 @@
   <mergeCells count="1">
     <mergeCell ref="B2:D2"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="B62"/>
-  </hyperlinks>
   <printOptions gridLines="1" horizontalCentered="1"/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.25" right="0.25" top="0.75"/>
   <pageSetup paperSize="9" cellComments="atEnd" orientation="landscape" pageOrder="overThenDown"/>
@@ -1871,9 +1872,7 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="1"/>
-      <c r="B29" s="23" t="s">
-        <v>49</v>
-      </c>
+      <c r="B29" s="23"/>
       <c r="C29" s="4"/>
       <c r="D29" s="5"/>
       <c r="E29" s="5"/>
@@ -1902,10 +1901,6 @@
       <formula1>"We need to spend more time to agree,We do not fully agree but will make it work,We fully agree"</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="C7"/>
-    <hyperlink r:id="rId2" ref="B29"/>
-  </hyperlinks>
   <printOptions gridLines="1" horizontalCentered="1"/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.25" right="0.25" top="0.75"/>
   <pageSetup paperSize="9" cellComments="atEnd" orientation="landscape" pageOrder="overThenDown"/>

</xml_diff>